<commit_message>
Update gold data automatically
</commit_message>
<xml_diff>
--- a/data/gold_data.xlsx
+++ b/data/gold_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1645"/>
+  <dimension ref="A1:I1646"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44855,6 +44855,33 @@
       </c>
       <c r="I1645" t="inlineStr"/>
     </row>
+    <row r="1646">
+      <c r="A1646" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B1646" t="n">
+        <v>4498.7001953125</v>
+      </c>
+      <c r="C1646" t="n">
+        <v>4510.5</v>
+      </c>
+      <c r="D1646" t="n">
+        <v>4374.10009765625</v>
+      </c>
+      <c r="E1646" t="n">
+        <v>4392.39990234375</v>
+      </c>
+      <c r="F1646" t="n">
+        <v>170992</v>
+      </c>
+      <c r="G1646" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1646" t="n">
+        <v>0</v>
+      </c>
+      <c r="I1646" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>